<commit_message>
Begonnen met de navigatie op de ACME website
</commit_message>
<xml_diff>
--- a/Data/Config.xlsx
+++ b/Data/Config.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="23929"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="24326"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://uipath-my.sharepoint.com/personal/alexandra_veizu_uipath_com/Documents/Documents/Projects/FrameworkTemplates/REFramework/VB/Data/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\51059992\OneDrive - Adecco\Documenten\UiPath\AssignmentTristan\Data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="1" documentId="13_ncr:1_{00D541BD-CB78-4D75-8532-9AD73E8C785E}" xr6:coauthVersionLast="46" xr6:coauthVersionMax="46" xr10:uidLastSave="{F8C54E24-BA5C-4BF9-8DAB-2778512EC11B}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{848021BF-F060-4D6E-979C-0E336A4C1807}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-10248" yWindow="17508" windowWidth="21252" windowHeight="9444" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-16320" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Settings" sheetId="1" r:id="rId1"/>
@@ -22,7 +22,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="49" uniqueCount="45">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="58" uniqueCount="54">
   <si>
     <t>Name</t>
   </si>
@@ -160,6 +160,33 @@
   </si>
   <si>
     <t>ProcessABCQueue</t>
+  </si>
+  <si>
+    <t>ACME_URL</t>
+  </si>
+  <si>
+    <t>https://acme-test.uipath.com/login</t>
+  </si>
+  <si>
+    <t>URL ACME website</t>
+  </si>
+  <si>
+    <t>LoginACME</t>
+  </si>
+  <si>
+    <t>guillermo.lisapaly@modis.com</t>
+  </si>
+  <si>
+    <t>Login ACME website</t>
+  </si>
+  <si>
+    <t>PasswordACME</t>
+  </si>
+  <si>
+    <t>Verhaal86!</t>
+  </si>
+  <si>
+    <t>Password ACME website</t>
   </si>
 </sst>
 </file>
@@ -223,10 +250,78 @@
     </xf>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle name="Normal" xfId="0" builtinId="0"/>
+    <cellStyle name="Standaard" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
+  <colors>
+    <indexedColors>
+      <rgbColor rgb="00000000"/>
+      <rgbColor rgb="00FFFFFF"/>
+      <rgbColor rgb="00FF0000"/>
+      <rgbColor rgb="0000FF00"/>
+      <rgbColor rgb="000000FF"/>
+      <rgbColor rgb="00FFFF00"/>
+      <rgbColor rgb="00FF00FF"/>
+      <rgbColor rgb="0000FFFF"/>
+      <rgbColor rgb="00000000"/>
+      <rgbColor rgb="00FFFFFF"/>
+      <rgbColor rgb="00FF0000"/>
+      <rgbColor rgb="0000FF00"/>
+      <rgbColor rgb="000000FF"/>
+      <rgbColor rgb="00FFFF00"/>
+      <rgbColor rgb="00FF00FF"/>
+      <rgbColor rgb="0000FFFF"/>
+      <rgbColor rgb="00800000"/>
+      <rgbColor rgb="00008000"/>
+      <rgbColor rgb="00000080"/>
+      <rgbColor rgb="00808000"/>
+      <rgbColor rgb="00800080"/>
+      <rgbColor rgb="00008080"/>
+      <rgbColor rgb="00C0C0C0"/>
+      <rgbColor rgb="00808080"/>
+      <rgbColor rgb="009999FF"/>
+      <rgbColor rgb="00993366"/>
+      <rgbColor rgb="00FFFFCC"/>
+      <rgbColor rgb="00CCFFFF"/>
+      <rgbColor rgb="00660066"/>
+      <rgbColor rgb="00FF8080"/>
+      <rgbColor rgb="000066CC"/>
+      <rgbColor rgb="00CCCCFF"/>
+      <rgbColor rgb="00000080"/>
+      <rgbColor rgb="00FF00FF"/>
+      <rgbColor rgb="00FFFF00"/>
+      <rgbColor rgb="0000FFFF"/>
+      <rgbColor rgb="00800080"/>
+      <rgbColor rgb="00800000"/>
+      <rgbColor rgb="00008080"/>
+      <rgbColor rgb="000000FF"/>
+      <rgbColor rgb="0000CCFF"/>
+      <rgbColor rgb="00CCFFFF"/>
+      <rgbColor rgb="00CCFFCC"/>
+      <rgbColor rgb="00FFFF99"/>
+      <rgbColor rgb="0099CCFF"/>
+      <rgbColor rgb="00FF99CC"/>
+      <rgbColor rgb="00CC99FF"/>
+      <rgbColor rgb="00FFCC99"/>
+      <rgbColor rgb="003366FF"/>
+      <rgbColor rgb="0033CCCC"/>
+      <rgbColor rgb="0099CC00"/>
+      <rgbColor rgb="00FFCC00"/>
+      <rgbColor rgb="00FF9900"/>
+      <rgbColor rgb="00FF6600"/>
+      <rgbColor rgb="00666699"/>
+      <rgbColor rgb="00969696"/>
+      <rgbColor rgb="00003366"/>
+      <rgbColor rgb="00339966"/>
+      <rgbColor rgb="00003300"/>
+      <rgbColor rgb="00333300"/>
+      <rgbColor rgb="00993300"/>
+      <rgbColor rgb="00993366"/>
+      <rgbColor rgb="00333399"/>
+      <rgbColor rgb="00333333"/>
+    </indexedColors>
+  </colors>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
       <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
@@ -239,7 +334,7 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Kantoorthema">
   <a:themeElements>
     <a:clrScheme name="Office">
       <a:dk1>
@@ -536,12 +631,12 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:Z998"/>
-  <sheetFormatPr defaultColWidth="14.44140625" defaultRowHeight="15" customHeight="1"/>
+  <sheetFormatPr defaultColWidth="14.42578125" defaultRowHeight="15" customHeight="1"/>
   <cols>
-    <col min="1" max="1" width="43.5546875" customWidth="1"/>
+    <col min="1" max="1" width="43.5703125" customWidth="1"/>
     <col min="2" max="2" width="43" customWidth="1"/>
-    <col min="3" max="3" width="81.44140625" customWidth="1"/>
-    <col min="4" max="26" width="8.6640625" customWidth="1"/>
+    <col min="3" max="3" width="81.42578125" customWidth="1"/>
+    <col min="4" max="26" width="8.7109375" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:26" ht="14.25" customHeight="1">
@@ -589,7 +684,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="3" spans="1:26" ht="43.2">
+    <row r="3" spans="1:26" ht="45">
       <c r="A3" s="2" t="s">
         <v>31</v>
       </c>
@@ -599,7 +694,7 @@
       </c>
     </row>
     <row r="4" spans="1:26" ht="14.25" customHeight="1"/>
-    <row r="5" spans="1:26" ht="28.8">
+    <row r="5" spans="1:26" ht="30">
       <c r="A5" t="s">
         <v>20</v>
       </c>
@@ -610,9 +705,39 @@
         <v>23</v>
       </c>
     </row>
-    <row r="6" spans="1:26" ht="14.25" customHeight="1"/>
-    <row r="7" spans="1:26" ht="14.25" customHeight="1"/>
-    <row r="8" spans="1:26" ht="14.25" customHeight="1"/>
+    <row r="6" spans="1:26" ht="14.25" customHeight="1">
+      <c r="A6" t="s">
+        <v>45</v>
+      </c>
+      <c r="B6" t="s">
+        <v>46</v>
+      </c>
+      <c r="C6" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="7" spans="1:26" ht="14.25" customHeight="1">
+      <c r="A7" t="s">
+        <v>48</v>
+      </c>
+      <c r="B7" t="s">
+        <v>49</v>
+      </c>
+      <c r="C7" s="4" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="8" spans="1:26" ht="14.25" customHeight="1">
+      <c r="A8" t="s">
+        <v>51</v>
+      </c>
+      <c r="B8" t="s">
+        <v>52</v>
+      </c>
+      <c r="C8" t="s">
+        <v>53</v>
+      </c>
+    </row>
     <row r="9" spans="1:26" ht="14.25" customHeight="1"/>
     <row r="10" spans="1:26" ht="14.25" customHeight="1"/>
     <row r="11" spans="1:26" ht="14.25" customHeight="1"/>
@@ -1613,12 +1738,12 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:Z988"/>
-  <sheetFormatPr defaultColWidth="14.44140625" defaultRowHeight="15" customHeight="1"/>
+  <sheetFormatPr defaultColWidth="14.42578125" defaultRowHeight="15" customHeight="1"/>
   <cols>
     <col min="1" max="1" width="41" customWidth="1"/>
     <col min="2" max="2" width="51" customWidth="1"/>
-    <col min="3" max="3" width="75.44140625" customWidth="1"/>
-    <col min="4" max="26" width="8.6640625" customWidth="1"/>
+    <col min="3" max="3" width="75.42578125" customWidth="1"/>
+    <col min="4" max="26" width="8.7109375" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:26" ht="14.25" customHeight="1">
@@ -1655,7 +1780,7 @@
       <c r="Y1" s="1"/>
       <c r="Z1" s="1"/>
     </row>
-    <row r="2" spans="1:26" ht="28.8">
+    <row r="2" spans="1:26" ht="30">
       <c r="A2" t="s">
         <v>5</v>
       </c>
@@ -1666,7 +1791,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="3" spans="1:26" ht="43.2">
+    <row r="3" spans="1:26" ht="45">
       <c r="A3" t="s">
         <v>33</v>
       </c>
@@ -1780,7 +1905,7 @@
       </c>
     </row>
     <row r="16" spans="1:26" ht="14.25" customHeight="1"/>
-    <row r="17" spans="1:3" ht="28.8">
+    <row r="17" spans="1:3" ht="45">
       <c r="A17" t="s">
         <v>40</v>
       </c>
@@ -2771,12 +2896,12 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
   <dimension ref="A1:Z1000"/>
-  <sheetFormatPr defaultColWidth="14.44140625" defaultRowHeight="15" customHeight="1"/>
+  <sheetFormatPr defaultColWidth="14.42578125" defaultRowHeight="15" customHeight="1"/>
   <cols>
-    <col min="1" max="1" width="31.88671875" customWidth="1"/>
-    <col min="2" max="2" width="30.109375" customWidth="1"/>
-    <col min="3" max="3" width="60.33203125" customWidth="1"/>
-    <col min="4" max="26" width="65.44140625" customWidth="1"/>
+    <col min="1" max="1" width="31.85546875" customWidth="1"/>
+    <col min="2" max="2" width="30.140625" customWidth="1"/>
+    <col min="3" max="3" width="60.28515625" customWidth="1"/>
+    <col min="4" max="26" width="65.42578125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:26" ht="14.25" customHeight="1">

</xml_diff>

<commit_message>
Dispatcher aangemaakt, CloseAllApps & KillAllProcesses aangepast
</commit_message>
<xml_diff>
--- a/Data/Config.xlsx
+++ b/Data/Config.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\51059992\OneDrive - Adecco\Documenten\UiPath\AssignmentTristan\Data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{109B0C05-CEF4-4011-94AB-01F250B0616C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{78827320-3FB6-4E81-88E5-9260E6F98BCE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -165,9 +165,6 @@
     <t>ACME_URL</t>
   </si>
   <si>
-    <t>https://acme-test.uipath.com/login</t>
-  </si>
-  <si>
     <t>URL ACME website</t>
   </si>
   <si>
@@ -186,7 +183,10 @@
     <t>Password ACME website</t>
   </si>
   <si>
-    <t>New System.Net.NetworkCredential("","b:HLGXL!3uk-8WA").SecurePassword</t>
+    <t>b:HLGXL!3uk-8WA</t>
+  </si>
+  <si>
+    <t>https://acme-test.uipath.com/</t>
   </si>
 </sst>
 </file>
@@ -238,7 +238,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
@@ -248,6 +248,7 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Standaard" xfId="0" builtinId="0"/>
@@ -641,33 +642,33 @@
       <c r="A6" t="s">
         <v>45</v>
       </c>
-      <c r="B6" t="s">
+      <c r="B6" s="5" t="s">
+        <v>53</v>
+      </c>
+      <c r="C6" t="s">
         <v>46</v>
-      </c>
-      <c r="C6" t="s">
-        <v>47</v>
       </c>
     </row>
     <row r="7" spans="1:26" ht="14.25" customHeight="1">
       <c r="A7" t="s">
+        <v>47</v>
+      </c>
+      <c r="B7" t="s">
         <v>48</v>
       </c>
-      <c r="B7" t="s">
+      <c r="C7" s="4" t="s">
         <v>49</v>
-      </c>
-      <c r="C7" s="4" t="s">
-        <v>50</v>
       </c>
     </row>
     <row r="8" spans="1:26" ht="14.25" customHeight="1">
       <c r="A8" t="s">
+        <v>50</v>
+      </c>
+      <c r="B8" t="s">
+        <v>52</v>
+      </c>
+      <c r="C8" t="s">
         <v>51</v>
-      </c>
-      <c r="B8" t="s">
-        <v>53</v>
-      </c>
-      <c r="C8" t="s">
-        <v>52</v>
       </c>
     </row>
     <row r="9" spans="1:26" ht="14.25" customHeight="1"/>

</xml_diff>